<commit_message>
Added file to rewrite implan codes that generated errors when running county and district models in IMPLAN. Accorindgly ran lines 98 onwards of the master analysis code to generate updated activity sheets. Also updated SmartPay file for FY2025 SmartPay data.
</commit_message>
<xml_diff>
--- a/data/raw/SmartPay.xlsx
+++ b/data/raw/SmartPay.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sumeet.bedi\Documents\R\meis_code\meis_pre-implan_activity_sheets\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5D1747E-E5B4-405F-B849-1EE2D3782EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF3187F8-8C16-4E6A-BC7E-622241097EDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14610" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28740" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Counties" sheetId="4" r:id="rId1"/>
@@ -602,14 +602,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C59"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.15625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.1796875" customWidth="1"/>
-    <col min="3" max="3" width="19.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.15625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.15625" customWidth="1"/>
+    <col min="3" max="3" width="19.7890625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>58</v>
       </c>
@@ -620,18 +620,18 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>31230581.619265374</v>
+        <v>30108587.369598612</v>
       </c>
       <c r="C2">
-        <v>1144613321.1833079</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1180506309.5359502</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -639,483 +639,483 @@
         <v>0</v>
       </c>
       <c r="C3">
-        <v>1175843902.8025732</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210614896.9055488</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4">
-        <v>16858.804255874671</v>
+        <v>16306.500123961567</v>
       </c>
       <c r="C4">
-        <v>1175827043.9983172</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210598590.4054248</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5">
-        <v>495078.98372410901</v>
+        <v>470137.01411941042</v>
       </c>
       <c r="C5">
-        <v>1175348823.8188491</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210144759.8914294</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6">
-        <v>38626.052847391256</v>
+        <v>35836.920668678795</v>
       </c>
       <c r="C6">
-        <v>1175805276.7497258</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210579059.9848802</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7">
-        <v>25763.027784246624</v>
+        <v>23927.518293227396</v>
       </c>
       <c r="C7">
-        <v>1175818139.7747889</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210590969.3872557</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8">
-        <v>6569819.3423523987</v>
+        <v>6281974.6166187823</v>
       </c>
       <c r="C8">
-        <v>1169274083.4602208</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1204332922.2889299</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9">
-        <v>126342.95909462948</v>
+        <v>130261.3727715593</v>
       </c>
       <c r="C9">
-        <v>1175717559.8434787</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210484635.5327773</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10">
-        <v>428108.98576368834</v>
+        <v>403800.23968835094</v>
       </c>
       <c r="C10">
-        <v>1175415793.8168094</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210211096.6658604</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11">
-        <v>34833223.066568404</v>
+        <v>38412489.299941063</v>
       </c>
       <c r="C11">
-        <v>1141010679.7360048</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1172202407.6056077</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12">
-        <v>27078.544764719627</v>
+        <v>25123.241672933837</v>
       </c>
       <c r="C12">
-        <v>1175816824.2578084</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210589773.6638758</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1173138.4743443225</v>
+        <v>1201042.5036986736</v>
       </c>
       <c r="C13">
-        <v>1174670764.328229</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209413854.4018502</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14">
-        <v>2802275.074220045</v>
+        <v>2885205.330289098</v>
       </c>
       <c r="C14">
-        <v>1173041627.7283533</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1207729691.5752597</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15">
-        <v>28581.349580856411</v>
+        <v>26517.531096944702</v>
       </c>
       <c r="C15">
-        <v>1175815321.4529924</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210588379.3744519</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B16">
-        <v>6872728.6444133827</v>
+        <v>6400353.7116875118</v>
       </c>
       <c r="C16">
-        <v>1168971174.1581597</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1204214543.1938612</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17">
-        <v>388844.68191649916</v>
+        <v>360898.0849436642</v>
       </c>
       <c r="C17">
-        <v>1175455058.1206567</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210253998.820605</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18">
-        <v>153263.86405088831</v>
+        <v>142196.89904809446</v>
       </c>
       <c r="C18">
-        <v>1175690638.9385223</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210472700.0065007</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19">
-        <v>59687.673593876534</v>
+        <v>55377.711824008271</v>
       </c>
       <c r="C19">
-        <v>1175784215.1289794</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210559519.1937249</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20">
-        <v>261080438.21793818</v>
+        <v>270333820.20356399</v>
       </c>
       <c r="C20">
-        <v>914763464.58463502</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+        <v>940281076.70198488</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21">
-        <v>109167.53318797336</v>
+        <v>102946.64620090819</v>
       </c>
       <c r="C21">
-        <v>1175734735.2693853</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210511950.2593479</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22">
-        <v>1677025.0344055218</v>
+        <v>1602676.7197813825</v>
       </c>
       <c r="C22">
-        <v>1174166877.7681677</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209012220.1857674</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B23">
-        <v>30666.755554197218</v>
+        <v>29414.294524533638</v>
       </c>
       <c r="C23">
-        <v>1175813236.047019</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210585482.6110244</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B24">
-        <v>349569.06011458929</v>
+        <v>339501.58336650929</v>
       </c>
       <c r="C24">
-        <v>1175494333.7424586</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210275395.3221824</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B25">
-        <v>382921.72925475793</v>
+        <v>411362.50041749503</v>
       </c>
       <c r="C25">
-        <v>1175460981.0733185</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210203534.4051313</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B26">
-        <v>2861.1086094549119</v>
+        <v>2654.5120379400742</v>
       </c>
       <c r="C26">
-        <v>1175841041.6939638</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210612242.3935108</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B27">
-        <v>2747.1105553311572</v>
+        <v>2548.745620694242</v>
       </c>
       <c r="C27">
-        <v>1175841155.6920178</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210612348.1599281</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B28">
-        <v>5960268.7070061238</v>
+        <v>5572501.6481917007</v>
       </c>
       <c r="C28">
-        <v>1169883634.095567</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1205042395.2573571</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B29">
-        <v>2987822.6329150884</v>
+        <v>2824179.0013087755</v>
       </c>
       <c r="C29">
-        <v>1172856080.1696582</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1207790717.9042401</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B30">
-        <v>442932.47901938146</v>
+        <v>428774.26829439477</v>
       </c>
       <c r="C30">
-        <v>1175400970.3235538</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210186122.6372545</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31">
-        <v>76298087.575038344</v>
+        <v>71878132.971550182</v>
       </c>
       <c r="C31">
-        <v>1099545815.2275348</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1138736763.9339986</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B32">
-        <v>18768414.834343832</v>
+        <v>17569583.32727297</v>
       </c>
       <c r="C32">
-        <v>1157075487.9682293</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1193045313.5782759</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33">
-        <v>24423.59024372026</v>
+        <v>22699.583706708127</v>
       </c>
       <c r="C33">
-        <v>1175819479.2123294</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210592197.3218422</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B34">
-        <v>11907101.909557194</v>
+        <v>11445179.680365449</v>
       </c>
       <c r="C34">
-        <v>1163936800.8930161</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1199169717.2251832</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B35">
-        <v>99394698.369245455</v>
+        <v>109239206.09515484</v>
       </c>
       <c r="C35">
-        <v>1076449204.4333277</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1101375690.810394</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B36">
-        <v>71840.915025681839</v>
+        <v>67249.453685508459</v>
       </c>
       <c r="C36">
-        <v>1175772061.8875475</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210547647.4518633</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B37">
-        <v>83339205.107593536</v>
+        <v>90687501.450804561</v>
       </c>
       <c r="C37">
-        <v>1092504697.6949797</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1119927395.4547443</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B38">
-        <v>227264376.36503679</v>
+        <v>228243564.4891448</v>
       </c>
       <c r="C38">
-        <v>948579526.43753648</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+        <v>982371332.41640401</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B39">
-        <v>78922457.751540005</v>
+        <v>86689829.38814266</v>
       </c>
       <c r="C39">
-        <v>1096921445.0510333</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1123925067.5174062</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B40">
-        <v>1085812.2799584353</v>
+        <v>1031587.1194136729</v>
       </c>
       <c r="C40">
-        <v>1174758090.5226147</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209583309.7861352</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B41">
-        <v>2623135.2537223031</v>
+        <v>2491889.9332979163</v>
       </c>
       <c r="C41">
-        <v>1173220767.548851</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1208123006.9722509</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B42">
-        <v>9293503.8612348735</v>
+        <v>8940836.0128587671</v>
       </c>
       <c r="C42">
-        <v>1166550398.9413383</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1201674060.8926899</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B43">
-        <v>11179368.236918135</v>
+        <v>10479473.299906775</v>
       </c>
       <c r="C43">
-        <v>1164664534.565655</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1200135423.6056421</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B44">
-        <v>141625477.89687458</v>
+        <v>150119289.55830845</v>
       </c>
       <c r="C44">
-        <v>1034218424.9056987</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1060495607.3472403</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B45">
-        <v>3650475.5010937043</v>
+        <v>3560977.154056326</v>
       </c>
       <c r="C45">
-        <v>1172193427.3014796</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1207053919.7514925</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B46">
-        <v>708671.54697854258</v>
+        <v>674828.41449804453</v>
       </c>
       <c r="C46">
-        <v>1175135231.2555947</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209940068.4910507</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -1123,139 +1123,139 @@
         <v>0</v>
       </c>
       <c r="C47">
-        <v>1175843902.8025732</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210614896.9055488</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B48">
-        <v>56122.806394795574</v>
+        <v>53692.295422152776</v>
       </c>
       <c r="C48">
-        <v>1175787779.9961784</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210561204.6101267</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B49">
-        <v>10339010.13558059</v>
+        <v>9776473.160012722</v>
       </c>
       <c r="C49">
-        <v>1165504892.6669927</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1200838423.7455361</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B50">
-        <v>7032965.5724888463</v>
+        <v>7014439.2499110885</v>
       </c>
       <c r="C50">
-        <v>1168810937.2300844</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1203600457.6556377</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B51">
-        <v>1714817.6931104304</v>
+        <v>1674037.9452338393</v>
       </c>
       <c r="C51">
-        <v>1174129085.1094627</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1208940858.960315</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B52">
-        <v>1739125.1494576042</v>
+        <v>1644057.7382129731</v>
       </c>
       <c r="C52">
-        <v>1174104777.6531155</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1208970839.1673357</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B53">
-        <v>3384.1399970509337</v>
+        <v>3224.3609630635469</v>
       </c>
       <c r="C53">
-        <v>1175840518.6625762</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210611672.5445857</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B54">
-        <v>962.09506699422286</v>
+        <v>892.62355456876026</v>
       </c>
       <c r="C54">
-        <v>1175842940.7075062</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210614004.2819943</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B55">
-        <v>964244.75116341154</v>
+        <v>923648.73635104951</v>
       </c>
       <c r="C55">
-        <v>1174879658.0514097</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209691248.1691978</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B56">
-        <v>29154.849696931</v>
+        <v>27332.546550451159</v>
       </c>
       <c r="C56">
-        <v>1175814747.9528763</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1210587564.3589983</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B57">
-        <v>26022407.934492663</v>
+        <v>24479560.707236759</v>
       </c>
       <c r="C57">
-        <v>1149821494.8680806</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1186135336.198312</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B58">
-        <v>1014399.33635569</v>
+        <v>949120.27548315492</v>
       </c>
       <c r="C58">
-        <v>1174829503.4662175</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+        <v>1209665776.6300657</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B59">
-        <v>2473835.8272620304</v>
+        <v>2296173.3450565129</v>
       </c>
       <c r="C59">
-        <v>1173370066.9753113</v>
+        <v>1208318723.5604923</v>
       </c>
     </row>
   </sheetData>
@@ -1266,12 +1266,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B53"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="2" max="2" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.7890625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>61</v>
       </c>
@@ -1279,420 +1279,420 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>5394397.5657269405</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+        <v>5065233.1631570589</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>6395895.0093248095</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+        <v>6349562.4510038421</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>20134171.959674578</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+        <v>18865577.420919523</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>7837672.5056108553</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+        <v>7602255.9374995427</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>2250252.2570443386</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2177924.830122503</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>95695605.088141605</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+        <v>105700607.62068118</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3369887.4607956312</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3240871.3005778068</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>13868462.76968069</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+        <v>13084587.76901301</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1003465.8851291446</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+        <v>953270.40182511241</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>4359878.9480833113</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4234644.3996717744</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>78591389.565920576</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+        <v>86357390.6693611</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
-        <v>8565929.7518094163</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+        <v>8332933.844470541</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>1003153.0628867242</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+        <v>1000778.9569698811</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>13335913.575441713</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+        <v>12788585.788161779</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
-        <v>6562058.6444491139</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+        <v>6337066.9953830652</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>111519082.85849249</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+        <v>121563804.58490109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
-        <v>34066318.882204346</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+        <v>32483044.24894236</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19">
-        <v>6100212.8598425156</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+        <v>5814610.2124264212</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20">
-        <v>11099160.824633928</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+        <v>10472562.904557187</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21">
-        <v>5263967.8674285579</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4915003.1419224311</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22">
-        <v>34470335.693818867</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+        <v>38080090.850769281</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23">
-        <v>842122.34656818339</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+        <v>790053.07809746847</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24">
-        <v>5488477.513278069</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+        <v>5124940.2546495823</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25">
-        <v>14159422.570321985</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+        <v>13368299.756986836</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26">
-        <v>3581952.7949114544</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3628453.8560580835</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
-        <v>28050027.060197592</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+        <v>26416067.13911587</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28">
-        <v>7653316.16149427</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+        <v>7283782.0692582559</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29">
-        <v>9084012.2919044383</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+        <v>8746269.8335244227</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
-        <v>37397933.575277612</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+        <v>40673734.017310895</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
-        <v>3933558.6490598358</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+        <v>3750749.0014678417</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32">
-        <v>12021898.321771592</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+        <v>11537743.529280853</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33">
-        <v>51790844.605490699</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+        <v>54679962.021914512</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34">
-        <v>1602102.560576146</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+        <v>1553854.4186323173</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35">
-        <v>2927773.740504209</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+        <v>2767088.6289163833</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36">
-        <v>4539748.4016295914</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4325377.1427937662</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37">
-        <v>21099810.632122565</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+        <v>20464282.015512876</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38">
-        <v>6691800.7370710149</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+        <v>6315835.0821407828</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39">
-        <v>8856414.1306743454</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+        <v>8386664.2022059299</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40">
-        <v>5117565.9377806</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4940582.2116758777</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41">
-        <v>21419735.326439861</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+        <v>20131860.796382524</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42">
-        <v>4399841.3754453873</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+        <v>4191326.3134603603</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43">
-        <v>78751584.018839538</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+        <v>85411404.910951912</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44">
-        <v>11047212.749107674</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+        <v>10661344.47351863</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45">
-        <v>6720862.4091839427</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+        <v>6590323.5901921708</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46">
-        <v>15669417.118760258</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+        <v>14757594.593669713</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47">
-        <v>9159824.9036921747</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+        <v>8650242.1956310607</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48">
-        <v>16501140.478247754</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+        <v>15736458.564543657</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49">
-        <v>12149536.409640877</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+        <v>11554429.627295738</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50">
-        <v>20599942.448814765</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+        <v>19396300.826531433</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51">
-        <v>130839378.90269767</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+        <v>137179902.40633935</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52">
-        <v>46368066.487292938</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+        <v>43688221.687985279</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.55000000000000004">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53">
-        <v>21626967.991034888</v>
+        <v>20556257.949222136</v>
       </c>
     </row>
   </sheetData>
@@ -1711,6 +1711,24 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="5aff56ac-f36b-49b3-8eea-e42fc37821cb">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <TaxCatchAll xmlns="5aff56ac-f36b-49b3-8eea-e42fc37821cb" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e750500f-42a5-4b8d-9659-3e1833e664de">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100553AAAAFA06B6240B39104FB8E692371" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="eba564f50e7d9022606b3f7bd7682fa4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e750500f-42a5-4b8d-9659-3e1833e664de" xmlns:ns3="5aff56ac-f36b-49b3-8eea-e42fc37821cb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4532e00170a7e1de3b425fa31ccfbcc5" ns2:_="" ns3:_="">
     <xsd:import namespace="e750500f-42a5-4b8d-9659-3e1833e664de"/>
@@ -1933,24 +1951,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="5aff56ac-f36b-49b3-8eea-e42fc37821cb">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <TaxCatchAll xmlns="5aff56ac-f36b-49b3-8eea-e42fc37821cb" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="e750500f-42a5-4b8d-9659-3e1833e664de">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29C5B0C8-44BE-460B-A97B-BA121A2B9D33}">
   <ds:schemaRefs>
@@ -1960,6 +1960,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6AEFC7D-86EA-49F2-A582-18F0D138CCEF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5aff56ac-f36b-49b3-8eea-e42fc37821cb"/>
+    <ds:schemaRef ds:uri="e750500f-42a5-4b8d-9659-3e1833e664de"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D39A3E9A-9507-4FCC-B661-F01599FA1F74}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1976,15 +1987,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A6AEFC7D-86EA-49F2-A582-18F0D138CCEF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5aff56ac-f36b-49b3-8eea-e42fc37821cb"/>
-    <ds:schemaRef ds:uri="e750500f-42a5-4b8d-9659-3e1833e664de"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>